<commit_message>
R3 层2：落 L2-31 名称截断+XSS、L2-28 ◆菱形SVG化+marker 14px
- L2-31：新增 esc()/truncateName() 公共函数，接入素材卡/特效卡/轨道标签/段头
  name 渲染（title 显示完整名），数据层字段零改动，顺带修素材名 XSS 注入
- L2-28：新增 kfDiamondSVG() 内联 SVG 菱形（fill/stroke 用 presentation attribute，
  便于 CSS .is-selected/.sel 覆盖状态），替换 kf-panel/audio-panel 文本 ◆；
  时间轴 .kf-marker 8→14px 内部插 SVG；面板 .kf-diamond div→SVG
- 验收总表追加 L2-31/L2-28 验收标准行（项目内 + 桌面两份 xlsx 同步）
- 纯前端无依赖，不碰 Api/draft schema/seg_id（L0-07 红线）

Co-Authored-By: WorkBuddy <workbuddy@tencent.com>
</commit_message>
<xml_diff>
--- a/docs/git-commit-log.xlsx
+++ b/docs/git-commit-log.xlsx
@@ -18,6 +18,8 @@
     <sheet name="M7 步骤索引" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="R3 步骤索引" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="R3 验收差距表" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="验收总表" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="已知Bug清单" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'提交记录'!$A$1:$F$25</definedName>
@@ -78,7 +80,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +119,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
       </patternFill>
     </fill>
   </fills>
@@ -181,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -263,6 +270,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2353,6 +2363,1554 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" style="3" min="1" max="1"/>
+    <col width="7" customWidth="1" style="3" min="2" max="2"/>
+    <col width="78" customWidth="1" style="3" min="3" max="3"/>
+    <col width="20" customWidth="1" style="3" min="4" max="4"/>
+    <col width="44" customWidth="1" style="3" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>卡号</t>
+        </is>
+      </c>
+      <c r="B1" s="26" t="inlineStr">
+        <is>
+          <t>层</t>
+        </is>
+      </c>
+      <c r="C1" s="26" t="inlineStr">
+        <is>
+          <t>验收标准（提取自卡片⑥，可测）</t>
+        </is>
+      </c>
+      <c r="D1" s="26" t="inlineStr">
+        <is>
+          <t>当前验收状态</t>
+        </is>
+      </c>
+      <c r="E1" s="26" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="130" customHeight="1" s="3">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>L0-01</t>
+        </is>
+      </c>
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C2" s="27" t="inlineStr">
+        <is>
+          <t>1. **计数器验收**：拖动片段 100px 持续 3 秒，在 `renderAll`/`renderPreview`/`drawAllWaves`/`renderRuler` 入口打点：三个函数调用次数均为 **0**。
+2. **跟手验收**：被拖段 `left` 在拖动中每帧更新、无"鼠标停了才跟上"；吸附命中时 `snapGuide` 竖线实时出现/消失。
+3. **落点验收**：拖动中 dropLine/dragLine/drop-target 轨高亮实时（依赖 L0-02；若 L0-02 未落，此项标注"待 L0-02"）。
+4. **提交验收**：松手后 `drag` 切片触发 `renderTimeline` 恰好 1 次；数据经后端 RPC 回填后 `refresh` 全量 1 次（L0-12 会再收口）。
+5. **回归验收**：resize 拖动、整组移动（`move_group`）、缩放、书签切换、2s 轮询均无白屏/错位；拖动中轮询不触发。
+6. **播放验收**：播放中拖动仍被 `isPlaying` 冻结逻辑覆盖（`:1243`），不回归。
+---</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E2" s="27" t="inlineStr">
+        <is>
+          <t>行为需真机验收</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="130" customHeight="1" s="3">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>L0-02</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C3" s="27" t="inlineStr">
+        <is>
+          <t>1. **落点实时**：拖动片段（轴内）3 秒内 `drop-target` 轨蓝框与 dropLine/dragLine 随 `curLeftUs`/`targetKind` 变化**实时更新**（打点：`updateDropIndicators` 每帧调用、视觉无滞后）。
+2. **标尺/标签零重建**：拖动 3 秒内 `renderRuler` 调用 = 0；`track-label` 删除+重建次数 = 0。
+3. **波形零重绘**：拖动 3 秒内 `drawAllWaves` 调用 = 0；松手 refresh 后恢复。
+4. **跨轨不重建**：拖动跨轨 3 秒内 `#tlContent` 内 `.track/.seg` 的 `remove()` 执行次数 = 0；松手后结构按提交结果正确收敛。
+5. **回归**：缩放（Ctrl+滚轮）、书签切换、静音/隐藏、选中切换、2s 轮询仍正常重建标尺/标签/波形；`TIMELINE_KEYED_DIFF=false` 回退全量仍可用。
+6. **与 L0-01 联合**：拖动中 `renderAll` = 0 次（L0-01 验收项）且落点线实时（本卡验收项）同时成立。
+---</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>行为需真机验收</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="130" customHeight="1" s="3">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>L0-03</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>1. **正式数据零污染**：Player 拖元素 100px 过程中，`Store.state.draft` 内目标 seg 的 `params.transform.positionX/Y` **全程不变**；松手提交后变为新值。
+2. **三方一致**：拖动中 Player 元素位置、时间轴 KF marker（若该属性有通道）、Inspector 输入框值**三者同步变化**（拖参、拖 marker、Player 拖元素三条路径各测一次）。
+3. **单条 undo**：一次手势松手后 undo 栈 +1（后端 `undo_stack.json.gz` 或 `main.py:1188` 栈长度可查）；连续拖 5 次 = 5 条。
+4. **取消零污染**：Esc/pointercancel 后正式数据 = 手势前；`discardPreview` 后三方回落到正式值。
+5. **轮询不弹回**：拖参过程中 2s 轮询触发不导致预览值回跳（`previewActive()` 守卫生效）。
+6. **回归**：离散操作（reset、toggle 打点、select）仍即时提交，无"必须松手才生效"的回退。
+---</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>行为需真机验收：Player/Inspector/时间轴三方连续交互一致性</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="130" customHeight="1" s="3">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>L0-04</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>1. 拖动 clip 按住 Shift，全程无 `snap-guide` 竖线出现；松开 Shift 恢复吸附（对照 `onPhMove:2407` 现状行为）。
+2. resize 左右手柄按住 Shift 无吸附；播放头 Shift 行为不回归（现状 `:2407` 保持）。
+3. 预览区拖动元素：中心/四边距画布中心/四边 ≤ 8 屏像素时吸附并（L1-06 落地后）显示白线；松手白线消失；Shift 拖过不吸。
+4. 旋转：在 0/90/180/270 ±5° 内松手，落库 `rotation` 为整 90°（经 `update_segment_transform`）；Shift 旋转可停在 87° 之类非整角度。
+5. 素材库拖入时间轴，`refresh()` 后落点段 `start % frameUs(30fps) === 0`。
+6. 性能：100 段 × 各 3 关键帧的工程，连续拖动 60 帧（1 秒），`getPoints` 全量重建次数 ≤ 2（首帧 + 数据变更帧），其余命中缓存。
+7. 阈值裁决落地：卡验收时在 `SnapEngine` 常量区能查到最终阈值表（时间轴/预览/旋转三行），与裁决结论一致。</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="130" customHeight="1" s="3">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>L0-05</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>1. 10 分钟、300 段工程：标尺 tick 元素数 &lt; 200（可视区 + buffer），且滚动时元素数保持恒定级（增量补删）。
+2. 快速 Ctrl+滚轮 10 次：最终 zoom 值与"一次性大滚轮"接近（指数平滑），无 step 跳变；`pps()` 单调变化无回跳。
+3. 缩放后播放头屏幕位置不变（与缩放前视口相对位置一致）。
+4. 重开应用：`pxPerSec/snapOn/rippleOn/scrollLeft` 恢复（localStorage 分支 A）；再次关闭不丢失。
+5. 播放中缩放：片段块/标尺/播放头三者同步无错位（回归 `repositionTimelineZoom` 现有行为）。
+6. 拖动中拖动片段：标尺不整树重建（Chrome Performance 面板记录 `renderRuler` 调用次数，拖动 60 帧中 ≤ 2 次全量，其余为增量/平移）。
+7. Q8/Q18 裁决落地：存储载体与 buffer 常量在代码中有单一注释锚点，与验收记录一致。</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="130" customHeight="1" s="3">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>L0-06</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>1. 播放头移出元素范围（&lt; start 或 &gt; start+duration）：该元素全部 KF 字段 ◆ 禁用（disabled + opacity-50），点击无动作；输入框编辑落库为 base 修改（`seg.transform` 变化、`seg.animations[path]` 的 keys 不变）。
+2. 播放头在元素内：有通道字段输入落 `add_keyframe`（keys 增/改）；无通道字段落 `update_segment_transform`（base）。
+3. 删光某一通道全部关键帧：删除操作前后，`renderPreview` 画面在同一播放头位置不跳变；`get_state` 返回中 `animations[path]` 消失、对应 `transform`/`params` base = 删除前解析值。
+4. 容差：播放头停在某帧 ±1 帧内，◆ 为命中态（蓝实心）；点击删除后该帧消失；与 ±1 帧外（≥2 帧）时 ◆ 为未命中态。
+5. 打帧帧对齐回归：任意路径 `add_keyframe` 落库 `t % 33333 === 0`。
+6. 撤销回归：打一帧→删光（回写 base）→ undo → 帧恢复且 base 回旧值；redo → 帧删且 base 为新值。</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>行为需真机验收</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="130" customHeight="1" s="3">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>L0-07</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>1. **回归全绿**：重做前端完成后，`mcp_server.py` 全部工具在既有回归脚本/`tests/` 下跑通，无一个因签名或返回结构变化而失败。
+2. **结构等键**：对同一草稿，重做前后 `get_state()` 返回的 JSON 顶层键与 `draft` 三桶 + canvas 键集合逐键相等（允许 `version`/`domain_version` 自然递增）。
+3. **双向互见**：Agent 写一条 `add_to_timeline`，重做后前端刷新可见且可选中；前端拖一个段，MCP `get_state` 能读到。
+4. **护栏生效**：若落契约自检脚本——`draft_state.json` 结构断言通过；`contract_snapshot.json` 无意外 diff（或 diff 均有对应决策记录）。
+5. **无越界提交**：R3 全部提交记录中，没有触碰 3.1 不可变清单任一条的改动（code review 可用清单逐条勾验）。
+6. **Q1/Q12 有决议**：两份待决在 L0-08 动工前各产出一次明确分支裁定并记录在案。
+---</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>护栏文档可跟踪</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="130" customHeight="1" s="3">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>L0-08</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>1. 用 `add_keyframe` 写一个含缓动字段（经 `update_keyframe` 可选参数写入）的关键帧，`get_state` 返回中原样保留 `segmentToNext/leftHandle/rightHandle` 字段（分支 A）。
+2. 打开**旧版** `draft_state.json`（animations 为空或仅 `{keys}` 无 type 字段）：面板/预览/时间轴 marker 全部正常，`kfVal` 按 scalar+linear 默认回退求值，无报错。
+3. discrete 类型：写入 `type:"discrete"` 通道（bool 值），`kfVal` 恒返回左帧值，不与前后帧 lerp。
+4. 惰性清理：删光某 path 全部 key 后，`get_state` 中该 path 条目消失（现状行为保持）。
+5. 三方时间口径：前端 `TimelineMapper.playheadLocal`、后端 `add_keyframe` 的 `t`、导出 `_apply_keyframes_to_segment` 对同一播放头得到同一 local 时间（对拍测试，M7-7c 铁律）。
+6. MCP 回归：`get_segment_detail`/`get_state` 返回形态与改造前相比，**外层 `animations` 的 path→dict 形态不变**（分支 A）；Agent 读取旧字段的既有调用全部通过。
+7. 分支 B 场景（若裁决为 B）：额外验收"旧文件迁移脚本"——旧 `{path:{keys}}` 能无损转换为 `{bindings,channels}`，且 undo 栈中旧快照可回放。</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>行为需真机验收</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="130" customHeight="1" s="3">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>L0-09</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>1. **漏点修复**：变速（speed 变化）后，`seg.animations` 所有 `keys[].t ≤ seg.duration`，grep 断言通过（当前变速路径 KF 可越界，修复后必不越界）。
+2. **一致性**：同一组写操作分别经「UI 路径（store.js call）→ Api.execute」与「MCP 路径（_exec）→ Api.execute」，两次 `get_state` 的 `draft` 相关段逐键相等。
+3. **主轨强制 0**：`move_segment`/`relocate_segment` 把段移入主轨（video ti=0）后，该段 `start==0` 恒成立。
+4. **空轨剪除**：删除某轨最后一段后，非 `persistent_empty` 的空轨被剪除；显式「+轨」创建的空轨不被误剪。
+5. **回归全绿**：`tests/` 中 trim/speed/scale/move 相关用例在管线改造后全绿（尤其 trim 右缩补帧、变速后 KF clamp 两个新增断言）。
+6. **幂等**：对同一段连续两次触发管线，第二次输出与第一次逐键相等（无累计漂移）。
+---</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>写后幂等规整，不改三桶组织</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="130" customHeight="1" s="3">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>L0-10</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>1. **工具可达**：MCP 连接后 `upsert_keyframe`（或决策选定的工具名）出现在工具清单；docstring 含 `path` 枚举与 `time_us` 语义。
+2. **写入一致**：同一段同一属性同一时间，Agent 调 `upsert_keyframe` 与前端拖菱形/点 toggle 各写一次，`seg.animations[path].keys` 落盘结果逐键相等（值、时间、插值方式）。
+3. **upsert 语义**：对同一 `(path,time_us)` 连续写两次不同 value，第二次覆盖第一次（keys 数不增）。
+4. **帧吸附与 clamp**：`time_us` 传负值或超 duration 时后端 clamp 后仍合法（`keys[].t ∈ [0,duration]`），与 `main.py:3915-3919` 现有行为一致。
+5. **回归全绿**：既有 23 个 MCP 工具在新增工具后回归全绿（签名快照 diff 无意外变更）。
+6. **读侧闭环**：`get_keyframes`（若采纳）返回与 `get_segment_detail().animations` 一致；Agent 可完成「读现状→打帧→读结果」闭环。
+---</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>行为需真机验收</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="130" customHeight="1" s="3">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>L0-11</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>1. **零 alert 残留**：R3 完成后 grep `alert(` 在 `工作台v0.8时间轴.html` **零命中**（`showFatal` 用 DOM 构建不依赖 alert，天然满足）。
+2. **toast 行为**：模拟一次「添加素材失败」，页面出现 bottom-right error toast，文案完整（含 `r.error` 原文），非阻塞（可继续操作），4~6s 自动消失；连续触发 5 次显示 5 条堆叠互不覆盖。
+3. **tooltip 替换**：hover 素材区 tab 出现自绘 tooltip（白底/深灰 + 三角箭头），原生 title 不弹出；延迟 ≤300ms；滚动/移出后消失。
+4. **遮罩 blur**：打开 `skillModal`/`presetModal`，背景呈轻模糊（blur≥4px）+ 低透明度，且原有打开/关闭/确认行为回归通过。
+5. **快捷键入口**：顶栏可打开 `ShortcutsDialog`，至少覆盖 `HTML:3235-3278` 全部键位分组展示。
+6. **降级横幅（按 Q11 裁定）**：若启用——横幅出现在 topbar 下方、可关闭且关闭后不再弹出；若不启用——`maybeShowDegradedBanner()` 存在但不产生 DOM（接口可测：调用后 `document.querySelector` 无匹配）。
+7. **无回归**：`showFatal` 链路在人为 `throw` 后仍显示诊断卡（含 stack）；`refresh()` 在 toast/dialog 打开期间按既有 Lock 语义暂停/补刷，无 DOM 竞态。
+---</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>行为需真机验收</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="130" customHeight="1" s="3">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>L0-12</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>层0</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>1. **一条手势一条 undo**：拖动片段 → 撤销 1 次回到拖动前（含位置+选中焦点）；连拖 3 次 → 连续撤销 3 次逐步回退，无"一步跳两格"。
+2. **空操作零污染**：单击片段（不拖动）→ undo 栈长度不变；拖回原位（|Δ|≤10ms）→ undo 栈长度不变（`:2058` didMove 生效）。
+3. **多命令手势单条 undo**：KF 组拖（一次拖多通道 KF）→ undo 1 次全部回退。
+4. **提交延迟**：松手到画面稳定 ≤ 1 个 RTT（RPC+refresh），无可见回填闪烁（L0-01/02 落地后全量重渲只发生 1 次）。
+5. **redo 与选中**：undo 后 redo 恢复手势后状态；undo/redo 后 `selectedKey/selectedKeys/selectedMaterialUid` 还原正确（`applySelection`）。
+6. **竞态回归**：提交后 2s 轮询不触发"撤销后又回来"；Agent 并发修改（MCP `execute`）与 UI undo 交互无异常。
+---</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>行为需真机验收</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="130" customHeight="1" s="3">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>L1-01</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>1. **纵向跟随**：拖动 video 段跨过下方 audio 轨（下移 ≥100px），拖动全程段 DOM 的 `transform` 含 `translate3d(0, &lt;delta&gt;, 0)` 且 `&lt;delta&gt;` 与 `clientY - startMouseY` 逐帧一致；段视觉离开源轨区域。
+2. **真实节点**：拖动中 `#tlContent .seg[data-segid="X"]` 数量恒为 1（无 ghost 副本）；段仍在源轨 `.track` 内（`el.parentElement` 不变）。
+3. **不重建**：拖动 3 秒内 `#tlContent` 内 `.track/.seg` 的 `remove()` 执行次数 = 0（与 L0-02 验收项 4 互锁）。
+4. **落点联动**（与 L0-02 联合）：拖动中 `drop-target` 轨蓝框高亮实时、`dropLine` 竖线实时；松手后 `refresh()` 段落库归位，无视觉跳变。
+5. **回归**：轴内横向拖动（`offsetY≈0`）行为与现状一致；resize 拖动无 transform；整组横向移动无纵向跟随（保持现状）；播放中拖动仍被 `isPlaying` 冻结逻辑覆盖（`工作台v0.8时间轴.html:1243`）。
+6. **可选增强验收**（若采档位 2）：`targetKind==="existing"` 且跨轨时，段顶最终停在目标轨顶部（`displayRowTopY(targetDisplayIndex)`），误差 ≤2px。
+---</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>行为真机</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="130" customHeight="1" s="3">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>L1-02</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>1. 拖动 video/audio/text 任意 clip 按住 Shift，全程无 `snap-guide` 竖线出现；段可停在 `x % frameUs !== 0` 的位置（`refresh()` 后 `start` 非整帧）；松开 Shift 吸附恢复。
+2. resize 左/右手柄按住 Shift：可拖到非吸附长度（`start+duration` 非整帧）；无竖线；松开恢复。
+3. 播放头拖动按住 Shift：行为与现状 `:2407` 完全一致（回归）；不出现"播放头吸到自己"抖动。
+4. `snapOn=false`（关闭吸附）时，Shift 按下与否均无竖线（回归）。
+5. `SnapEngine.isShiftDisabled` 在三路径（`:1938/:1963/:1985`）与播放头（`:2407`）共 4 处被一致调用（grep 验证无散落 `e.shiftKey` 字面判断）。
+6. 结合 Q4 裁决：若分支 B，`isShiftDisabled(e,{domain:"timeline"})` 与缩放侧锁比例语义并存无冲突（画布拖拽不受影响）。
+---</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="130" customHeight="1" s="3">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>L1-03</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>1. 空白区拖动：矩形在超激活阈值前**不显示**（或显示但无选区变化——按分支 B 实现则阈值 4px 内不显示）；超阈值后矩形显示。
+2. 拖动中矩形扫过的片段 `.sel` 描边**实时**亮起；矩形移出后对应片段 `.sel` 实时消失（对比现状：松手前无任何选中反馈）。
+3. 松手后 `Store.state.selectedKeys` = 最后一次矩形相交的 key 集合；`Store.set` 恰好 1 次（打点验证）。
+4. Shift 框选：拖动中实时并入既有选择（既有点不被取消）；松手后 `selectedKeys` = 既有 + 相交。
+5. 未超阈值（&lt;4px）点按空白：`selectKey(null)` 行为与现状一致（取消选中）。
+6. 框选中 2s 轮询不触发（`pendingBox` 守卫生效，打点 `refresh()` 调用 0 次）。
+7. 回归：松手后选中段可正常整组移动（`isGroup` 判定 `selectedKeys.length&gt;1` 不变，`工作台v0.8时间轴.html:1894`）。
+---</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>行为真机</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="130" customHeight="1" s="3">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>L1-04</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>1. **clip 拖动**：把被拖段拖到视口右缘 100px 内并停住 → `#tlScroll.scrollLeft` 自动增大（向右滚），速度随贴近边缘增大，单帧增量 ≤15px；被拖段与 `dropLine` 位置随内容同步移动（不脱节）；鼠标移出边缘带 → 停止。
+2. **播放头 scrub**：拖播放头到视口边缘 → 自动滚动追播放头；`playheadUs` 随滚动推进；与 `ensurePlayheadVisible` 不互相抢滚（无抖动/回跳）。
+3. **框选**：拖框选矩形到视口左缘 → 向左滚，矩形外扩，实时选中集随滚动扩展（L1-03 联动）。
+4. **停止**：任意交互 mouseup 后 `_edgeScrollCtx=null` 且 rAF 停止（`performance` 采样无持续 rAF 消耗）。
+5. **守卫**：边缘滚动期间 `ensurePlayheadVisible` 不触发抢滚；结束后 200ms 恢复原自动滚回行为。
+6. **回归**：无边缘滚动时（鼠标在视口中部）拖动/scrub/框选行为与现状完全一致；滚动不触发 `renderAll`（L0-01 打点验证调用 0 次）。
+---</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>行为真机</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="130" customHeight="1" s="3">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>L1-05</t>
+        </is>
+      </c>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>1. 拖播放头到某段起点/终点或书签 10px 阈值内：吸附命中瞬间手柄出现 `.snapped` class，边框实心 + 高亮（截图对比未吸附态差异明显）。
+2. 拖离吸附点、或按住 Shift 拖过吸附点：`.snapped` 消失（手柄回半透明边框）。
+3. 松手（`onPhUp`）：`.snapped` 与 `.dragging` 均被清理（无残留 class）。
+4. clip 拖动/resize 吸附命中（竖线出现）时：`#playheadHandle` 无 `.snapped` class（回归）。
+5. 手柄 hover 变亮与吸附实心共存：`.dragging.snapped` 时两种效果都可见（无一方被覆盖）。
+---</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="130" customHeight="1" s="3">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>L1-06</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>1. 拖动元素使元素左边（`中心x - 半宽`）靠近画布左边（`-W/2`）到 ≤ 8 屏像素：出现 `rgba(255,255,255,.7)` 1px 竖直贯穿线，元素被吸附到左边对齐；
+2. 元素中心靠近画布中心到 ≤ 8 屏像素：出现垂直+水平两条线（中心对齐），元素吸附到 (0,0)；
+3. 按住 Shift 拖过以上位置：**无线、不吸附**（元素停在原始 round 位置）；
+4. 松手：`#previewSnapGuides` 内容清空；`refresh()` 后元素位置 = 吸附值（`getProperty(seg,"transform.positionX")` 为整对齐值）；
+5. pointercancel（右键取消/窗口失焦）后同样无残留线；
+6. 缩放画布（zoom≠1）后重复 1-2：阈值仍为 **8 屏像素**（画布放大时逻辑吸附范围缩小，屏上表现为恒定 8px）；
+7. 回归：时间轴播放头拖动吸附蓝线（`HTML:2407-2411`）行为不变；预览元素拖动跟手（无 snap 时手感）不回归。
+---</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="130" customHeight="1" s="3">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>L1-07</t>
+        </is>
+      </c>
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>1. 旋转到 87°→吸附到 90°、92°→吸附到 90°、86°→不吸附（显示 86°）；179°→180°、181°→180°、184°→不吸附（184°）；270±5° 同理；
+2. 按住 Shift 旋转：87° 停在 87°、184° 停在 184°（全程不吸附）；
+3. 吸附松手后 `refresh()` 落库 `getProperty(seg,"transform.rotate")` = 整 90°（或 0）；undo 恢复拖前角；
+4. 吸附状态下包围盒与元素旋转角一致（截图对比无残差）；
+5. 回归：无吸附路径（Shift 按住 / 距离超阈值）与现状行为一致（`Math.round(...*10)/10` 精度保留）。
+---</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="130" customHeight="1" s="3">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>L1-08</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>1. 角点缩放：拖到 0.5/1.0/1.5/2.0 整数比例附近（阈值内）吸附；边点拖到整数单轴比例吸附；Shift 拖过不吸附；
+2. 有 `transform.scaleX/Y` 动画通道的段，拖角点缩放并松手：`refresh()` 后 `seg.animations` 中两个 path **消失**（分支 B 后端删除）或会话内消失（分支 A，见 ③3.2 分支差异），`transform.scaleX/Y` = 拖后静态值；
+3. 缩放下限：拖到极小，最小 scale = 0.01（不再停 0.05）；
+4. 拖后手柄包围盒与元素实际尺寸一致（截图对比无残差）；
+5. 回归：无动画通道段缩放行为不回归；undo 一次恢复拖前 scale 与（若分支 B）动画通道。
+---</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>缩放吸附 0.25/0.5/0.75/1/1.25/1.5/2/3/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="130" customHeight="1" s="3">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>L1-09</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>1. 对**有** X/Y 动画通道的段：播放头在段内拖动 100px 松手，`refresh()` 后 `seg.animations["transform.positionX"].keys.length` 与拖前**相等**；`seg.transform.x`（或 `params`）为拖后值；
+2. 对**无**通道段：base 值改变（不回归）；
+3. undo 栈：一次拖动 = +1 条（`drag-transform`，非 `drag-transform-kf`）；
+4. 替代打帧路径（分支 B）：修饰键 + 拖动产生关键帧（若裁决 B）；分支 A：仅 Inspector ◆/＋/时间轴 marker 可打帧；
+5. 回归：Inspector ◆/＋（`toggleKf :HTML:1679`、`addKfAtPlayhead :HTML:1703`）、时间轴 marker 拖动打帧（`HTML:2143-2230`）行为不变。
+---</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="130" customHeight="1" s="3">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>L1-10</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>1. **Player 拖元素**：按住拖动，Inspector X/Y 输入框值**实时**跟随（不松手即变）；松手提交后与最终值一致；
+2. **时间轴拖 KF marker**：拖动中 Player 元素位置/缩放**实时**按新 key 时间插值（无滞后）；Inspector 对应字段值实时；松手 marker 停在新位置，undo 一次回退；
+3. **Inspector 输入**（通道开）：输入中时间轴 KF marker **实时**移动（菱形左/右移）；松手/失焦后 marker 停在输入值位置；
+4. 以上三路径松手后**恰好 1 次提交 + 1 条 undo**；
+5. 拖中触发一次 2s 轮询：三方值不回跳（preview 态覆盖，刷新后仍显示拖中值）；
+6. 取消（Esc/pointercancel）：三方回落到手势前正式值（`discardPreview` 生效），无预览态残留。
+---</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>行为真机：参数拖中联动 Player/Inspector/时间轴</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="130" customHeight="1" s="3">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>L1-11</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>1. 快速拖动播放头 500ms（约 30 帧 move）：Player 画面 **每帧更新**（无 80ms 停顿窗口），肉眼无滞后；
+2. 播放头停在任意位置松手：`renderPreviewMaybe` 最后执行一次，Player 画面 = 播放头帧（帧对齐）；
+3. 拖动中播放头红线始终跟手（`positionPlayhead` 正常）；
+4. 播放头吸附（`snapOn` 开）行为不回归（蓝线 + 吸附值）；
+5. 松手 `onPhUp` 确定性 seek 后 undo/刷新正常（`Store.set` 一次）；
+6. 性能采样（验收报告附）：连续拖动 3 秒，`renderPreviewMaybe` 调用次数 ≤ 3 秒×60（rAF 上限）；`renderAll` 调用次数 = 0（拖动中）+ 1（松手）——证明 L0-01 收窄生效。
+---</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>机制落地</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>行为真机</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="130" customHeight="1" s="3">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>L1-12</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C25" s="27" t="inlineStr">
+        <is>
+          <t>1. 预览区 `Ctrl/Meta+滚轮`：`zoomPercent`（`HTML:500` `zoomPct`）连续变化，素材视图缩放，指数平滑无跳变；
+2. 时间轴缩放：分支 A 用 `Ctrl+Shift+滚轮` 或控制条按钮；分支 B 用 `Ctrl+滚轮`——均能让 `pxPerSec` 变化且以播放头为锚（`HTML:848-872`）；
+3. `HTML:494` title 与实际键位一致；
+4. `Shift+滚轮` 时间轴横向滚动（`HTML:3097-3100`）回归通过；
+5. 中键画布平移（`viewport-input.js:31-51`）回归通过；
+6. 画布缩放时 `syncZoomUI`（`HTML:3339-3342`）双向同步（按钮/滑块/百分比一致）。
+---</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="130" customHeight="1" s="3">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>L1-13</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>1. 预览画布空白处右键：弹菜单，含「适应屏幕/实际大小」，点击后 `zoomPct` 变化（fit→100%）；
+2. 预览画布内选中元素上右键：额外出现段级项（如「复制」），点击 `copy_to_buffer` 生效（粘贴可用）；
+3. 菜单外点击 / Esc：菜单关闭；
+4. 时间轴片段右键（`HTML:2818`）、标尺书签右键（`HTML:3050`）功能回归；
+5. 全屏/快照项按裁决分支显示为置灰或隐藏，且无 JS 报错；
+6. 拖动元素中按右键：不打断拖动、不弹菜单或弹菜单后拖动手势正确结束（pointerup 正常）。
+---</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="130" customHeight="1" s="3">
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>L1-14</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="inlineStr">
+        <is>
+          <t>1. 双击文字段：出现编辑外框 + 光标定位文字内容，`contentEditable="true"` 生效；
+2. 输入新内容：Player 预览实时更新（不松手即变）；
+3. blur（点击别处）：新内容提交（`refresh()` 后 `seg.text` = 新内容，undo +1）；无变化 blur 不产生 undo；
+4. Esc：丢弃本次修改，`seg.text` 保持编辑前（undo 不 +1）；
+5. 编辑中样式保持：字号/颜色/背景不变，仅内容变；
+6. 双击 video/image 元素：不进入文字编辑（仍选中/拖动）；
+7. 提交后导出 `main.py:2203` 读取的 `seg.text` = 新内容（DSL 一致性）。
+---</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>阻塞·待用户决策</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="inlineStr">
+        <is>
+          <t>需后端补 update_text 命令后再收口</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="130" customHeight="1" s="3">
+      <c r="A28" s="27" t="inlineStr">
+        <is>
+          <t>L1-15</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="inlineStr">
+        <is>
+          <t>1. 未旋转元素：分别悬停 l/r/t/b 边柄与 4 角柄、旋转柄，光标分别显示 `ew-resize/ns-resize/nwse-resize/nesw-resize/grab`；
+2. 元素旋转 45°：l/r 边柄光标变为 `ns-resize` 类方向（随角度），角柄 `nwse/nesw` 互换；
+3. 旋转柄拖动中光标 `grabbing`（按住状态）；
+4. 光标不闪烁（悬停稳定、拖动中不重建）；
+5. resize/rotate 手势功能（`ResizeSession`/`RotateSession`）回归通过，`data-h` 路由不变。
+---</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="130" customHeight="1" s="3">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>L1-16</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="inlineStr">
+        <is>
+          <t>1. 选中段手柄 **8 点**（无 top 边），旋转柄仍在 top 上方；
+2. 在视觉圆外 3px 内按下 → 命中并开始 resize（命中区 18px 生效）；
+3. 视觉圆本身按下 → 命中（视觉层 `pointer-events:none` 但被命中层覆盖）；
+4. zoom 放大 200% 后拖动素材，激活手感与 100% 时一致（逻辑像素口径，分支 A）或 3px 屏像素（分支 B）；
+5. 单击（未超阈值）仍走"仅选中"（`preview-drag.js:73`）；
+6. resize 角/边/旋转全手势回归（scaleX/scaleY/rotation 落库、undo 一条）。
+---</t>
+        </is>
+      </c>
+      <c r="D29" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="130" customHeight="1" s="3">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
+          <t>L1-17</t>
+        </is>
+      </c>
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="inlineStr">
+        <is>
+          <t>1. NumberField / speed / audio / KF 面板全部数字字段左侧出现 `cursor-ew-resize` icon；
+2. 按住 icon 拖 100px：值变化 = `100 × 0.5 × 单位换算`（slow 灵敏度），方向正确；
+3. 拖动中 Player 预览实时变化（transform/opacity/volume/effect 参数各自生效）；
+4. 拖动中 `Store.state.draft` 内目标 seg 的 `params`/`animations` **不变**（overlay 隔离）；松手后一次提交、undo +1；
+5. Esc / pointercancel：正式数据零变化（discardPreview）；
+6. 与输入路径共存：先点输入框再拖 icon 不串手势；Pointer Lock 降级路径（无锁）拖动手感可用；
+7. 多选批量（speed/audio `isBatch`）场景：scrub 仍走既有批量提交（`set_segments_props`），值实时刷全部段。
+---</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>阻塞·待用户决策</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>需立项 ScrubSession 前端新增（较大）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="130" customHeight="1" s="3">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>L1-18</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>1. 点击 NumberField/speed/audio/KF 面板输入框任意位置：全文选中（`selectionStart=0`、`selectionEnd=len`）；
+2. 全选后键入 `9`：旧值整体替换为 `9`（非插入）；
+3. 二次点击已聚焦输入框：仍全选（不取消选择、不放置 caret）；
+4. Enter → 提交；点击外部 → 提交；Escape → 分支 A 提交 / 分支 B 丢弃，均不产生二次提交（undo 栈 +1 或 +0 符合语义）；
+5. 提交后回显 clamp/step 规范化值（如 speed 输入 `99` 回显 `5`）；
+6. 播放头移动不吞输入（KF 面板）、面板切换不丢焦点（speed/audio 守卫回归）。
+---</t>
+        </is>
+      </c>
+      <c r="D31" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E31" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="130" customHeight="1" s="3">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>L1-19</t>
+        </is>
+      </c>
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>1. `1920/2` 失焦 → `960`；`100*1.5` → `150`；`50+50` → `100`（现状 50，修复点）；
+2. `-30`、`12.5`、`1e3` 走普通数值路径不误判；
+3. 表达式结果过 min/max → 钳制；非 step 倍数 → 吸附（如 step=10、`33/2=16.5` → 20）；
+4. `1+*2`、`abc`、`1920/` → 不采纳、原值保留、无 console 错误；
+5. KF 面板输入 `1920/2` 后点 `＋` 打点：落库 value=960（非字符串）；
+6. speed/audio/KF 面板表达式输入体验与 NumberField 一致。
+---</t>
+        </is>
+      </c>
+      <c r="D32" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="130" customHeight="1" s="3">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>L1-20</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>1. 拖动 effect 滑杆任意参数：预览画面实时变化（adjustment 作用栈滤镜 / clip 绑定段滤镜 / track 整轨），无 250ms 滞后；
+2. 拖动中 `Store.state.draft` 内 effect 段 `seg.params[pname]` **不变**（overlay 隔离，路线 A）；松手后一次 `update_effect` + `refresh`；
+3. undo 栈：拖一次 +1 条；
+4. 松手后画面/面板值 = 提交值（无回弹）；
+5. 拖动中切换选中段：无残留滤镜（discardPreview 生效）；
+6. 与 mask 滑杆（`mask-panel.js:122-127` 已实时）手感一致；effect 参数回调（`update_effect`）无重复调用。
+---</t>
+        </is>
+      </c>
+      <c r="D33" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E33" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="130" customHeight="1" s="3">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>L1-21</t>
+        </is>
+      </c>
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C34" s="27" t="inlineStr">
+        <is>
+          <t>1. **方向①（marker→Inspector）**：拖选中段 KF marker 越过播放头 → `kf-panel` 对应字段 ◆ 实时亮/灭，显示值随插值实时更新（拖动中无提交、无整面板重建）。
+2. **方向②（Inspector→marker）**：在 kf-panel 输入框拖动/逐键改值（`upsertLocal` 路径）→ 时间轴对应 `.kf-marker` 位置实时移动（`left` 随 t 变化），`renderTimeline` 不重建。
+3. **Player 同步（档位 A 验收）**：拖 KF marker 中 `renderPreview` 每帧渲染，Player 画面实时反映重定位后插值；打点 60fps 下主线程帧耗时 ≤ 16ms（超限则回退档位 B）。
+4. **松手纪律**：拖动全程 `update_keyframe` 调用 0 次；松手后 `withTx` 恰好 1 次事务、1 条 undo；`refresh()` 后数据与视觉一致。
+5. **轮询守卫**：KF 拖动中 2s 轮询 `refresh()` 不触发（`_kfDragActive` 守卫生效，打点 0 次）；松手后恢复。
+6. **回归**：单击 marker（未超 4px 阈值，`up :2208-2211`）仍 seek 播放头；Shift/Ctrl 多选组拖相对间隔保持（`session.deltaTicks` 单一值）；`withTx` 异常路径 `_kfDragActive` 释放（无锁死）。
+---</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E34" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="130" customHeight="1" s="3">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>L1-22</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>1. 在 kfGraph 拖任意菱形到任意位置松手：`get_state` 返回该 KF 的 `t % 33333 === 0`（30fps）。
+2. 拖动中菱形 `style.left` 随吸附后 t 跳动到整帧位置（打点 move 内 `t` 值恒整帧）。
+3. 拖动中 `update_keyframe` 调用 0 次；松手恰好 1 次（现状 up 提交语义保持）。
+4. 短段（duration &lt; 2 帧）拖动：落库 `t` 被 clamp 到 `[0, dur]` 且整帧，无越界/负值。
+5. 拖动 KF 到距既有帧 ≤1 帧处：松手后两端按容差合并/命中行为与 `KF_HIT_TOLERANCE_US`（`kf-channel.js:27`）一致，无"两帧差几微秒"脏状态。
+6. 回归：kfGraph 点选（`renderKfSel`）与时间轴 marker 拖动（`:2143`）不受影响；`kfSegArgs()` 提交参数不变。
+---</t>
+        </is>
+      </c>
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="130" customHeight="1" s="3">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
+          <t>L1-23</t>
+        </is>
+      </c>
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="inlineStr">
+        <is>
+          <t>1. 拖图片到已存在 video 段：该段 `opacity:.5`（`.drop-target-media` class 存在）；同时 `#dragLine`/`#clipGhost`/`#dropNewTrackHint` 均隐藏；轨道 `.drop-target` 不亮（互斥）。
+2. 拖到轨间隙（新建轨）：DragLine 通栏横线 + hint 显示（现状回归）；无元素高亮。
+3. 拖到已有轨空白：目标轨高亮 + DragLine（现状回归）。
+4. 拖 audio：全程无元素高亮（只落 audio 轨）。
+5. 拖 effect 到可绑定段：现有 `.drop-target-seg` 虚线环行为不回归（`:3134-3146`）。
+6. 松手命中元素（media）：出现「替换素材 coming soon」提示，不执行落轨；时间轴数据零变化（`get_state` 前后 diff 为空）。
+7. 拖动路径与松手路径同源：高亮元素与 drop 判定为同一段（对比 `__libDropCache.bindSeg` 与高亮 DOM `data-key`）。
+8. 回归：dragleave/drop 后所有指示 DOM 清理干净（无残留 class/线/hint），#516 风险面不扩大（轮询守卫无新增竞态）。
+---</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="130" customHeight="1" s="3">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>L1-24</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>层1</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>1. 素材库拖入时间轴任意位置：`refresh()` 后落点段 `start % TimelineMapper.frameUs(fps) === 0`（fps=30 时 `start % 33333 === 0`）；
+2. dragover 时影子段/落点线位置与 drop 实际落点段位置**一致**（同一帧吸附值，误差 &lt; 1px）；
+3. 特效拖入 bindTo 片段：`atTimeUs` 帧对齐（`% frameUs === 0`）；
+4. 拖到非整帧位置（如鼠标在 16ms 处）：落点停在 0ms 或 33ms（最近整帧），不落在 16ms；
+5. 回归：时间轴内已有段移动（move 路径）落点行为不变；播放头拖动吸附（`HTML:2407-2411`）不回归；
+6. 边界：拖到时间轴最左（0 附近）落点 `start=0`（`Math.max(0, ...)` 保留）；拖到末端落点不超过总时长（吸附值钳制）。
+---</t>
+        </is>
+      </c>
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>L2-28</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1. Inspector 所有 ◆ 按钮为 SVG 菱形（非文本字符）：有帧/播放头命中 → fill-primary 实心；未命中 → 灰/透明描边。
+2. 时间轴 .kf-marker 为 14×14px SVG 菱形：未选中白底黑边（strokeWidth 1.5）、选中 fill-primary；拖动/选中事件回归正常。
+3. 面板 KF 图 .kf-diamond 同 SVG 视觉，选中 .sel 高亮。
+4. 播放头出范围（L2-10 场景）→ ◆ 整体 opacity-50 且点击无效（禁用态视觉 + 门控回归）。
+5. audio 面板音量 ◆（audVolKf）同步 SVG 化。
+6. 无功能回归：toggleKf/startKfMarkerDrag/onKfDiamondDown 全链路正常。
+---</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>纯前端无依赖（C-6 视觉收尾）；kfDiamondSVG 用 presentation attribute 便于 CSS 覆盖状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>L2-31</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1. 素材卡：导入 &gt;16 字符文件名 → 卡片显示 前16+…+后3；≤16 字符 → 全名；hover 显示完整名。
+2. 拖入正确性：把该素材拖入时间轴 → 新段 s.name 为完整名（非截断）；hover「+」插入同理。
+3. 时间轴段名：长名段 .seg .hdr 显示截断文本，不溢出段边界，hover 见全名。
+4. 轨道标签：长轨道名 .track-label .name 以 … 结尾，hover 见全名。
+5. XSS 安全：文件名含 &lt;script&gt;/&amp; 字符 → 卡片名安全显示（转义），无注入；渲染不中断。
+6. 数据零改动：Store.state.materials[i].name 与 seg.name 保持原值（控制台断言）。
+---</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>纯前端无依赖；esc()+truncateName() 公共函数；数据层字段零改动，顺带修 XSS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="3" min="1" max="1"/>
+    <col width="34" customWidth="1" style="3" min="2" max="2"/>
+    <col width="30" customWidth="1" style="3" min="3" max="3"/>
+    <col width="9" customWidth="1" style="3" min="4" max="4"/>
+    <col width="22" customWidth="1" style="3" min="5" max="5"/>
+    <col width="14" customWidth="1" style="3" min="6" max="6"/>
+    <col width="52" customWidth="1" style="3" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>现象</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>关联模块·卡</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>严重度</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>发现日期</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
+          <t>根因·备注·牵连</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="96" customHeight="1" s="3">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>B-01</t>
+        </is>
+      </c>
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t>素材从素材库拖入时间轴，松手后回弹到原点（落点不保留）</t>
+        </is>
+      </c>
+      <c r="C2" s="27" t="inlineStr">
+        <is>
+          <t>时间轴拖拽落点 / timeline.js onDrop·addToTimeline·drop校验</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>阻断</t>
+        </is>
+      </c>
+      <c r="E2" s="27" t="inlineStr">
+        <is>
+          <t>未修</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="G2" s="27" t="inlineStr">
+        <is>
+          <t>疑既有#516拖素材清空类变体（回弹≠清空，属新观察）。落码前须grep落点校验定位『校验拒绝/落点被回填清』；素材拖拽路径与property drag不同，大概率无关本会话preview-state/snap改动，但须grep实证。P0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="96" customHeight="1" s="3">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>B-02</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="inlineStr">
+        <is>
+          <t>播放器跨段播放异常：MP3无声 / MP4卡顿 / drift死循环</t>
+        </is>
+      </c>
+      <c r="C3" s="27" t="inlineStr">
+        <is>
+          <t>player.js / media.js 媒体生命周期</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="inlineStr">
+        <is>
+          <t>重大</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>临时绕开(待彻底修复)</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-15(记忆)</t>
+        </is>
+      </c>
+      <c r="G3" s="27" t="inlineStr">
+        <is>
+          <t>Round A~E + B.5已收口媒体控制权(墙钟master + 跨段handoff)，但 seek/drag/pause-resume 仍乱；记忆记为『临时绕开方案』，未彻底修复。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="96" customHeight="1" s="3">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>B-03</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>拖素材清空（#516）：拖入素材偶发把时间轴清空</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>时间轴拖拽 / 刷新时序</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>待整段重做随OpenCut消失(不单修)</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>早期(记忆)</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>记忆决策：随R3整段重做消失，不单独修。专卡 L2-23 根治（须先 L0-01/L0-02 落地后专门排查）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="96" customHeight="1" s="3">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>B-04</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>关键帧 X/Y 通道漂移分离（X@95帧、Y@113帧）</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>kf-channel.js / property-kernel.js toggleKf</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>已记录待验(Phase1报告)</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>toggleKf 预览路径用实时播放头读数致通道漂移；Phase1时间轴对齐已落(12/12测试)。根因报告 kf-drag-problem-report-2026-08-21.md。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="96" customHeight="1" s="3">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>B-05</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>ui-feedback openDialog body 重复 append：字符串body不显示 / node body多空div</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>property/ui-feedback.js openDialog</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>已修(commit d1a3b7f 2026-08-27)</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>本会话已修：删多余 append 行，字符串body走textContent、node body走appendChild唯一一次。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
R3 验收总表补 A+C+D 三批卡（L2-01/02/04/05/06/07/09/10/18/23，R61-70）
- A组7：L2-02文本KF / L2-04 Graphic / L2-05缓动曲线 / L2-06 Scale组KF / L2-07颜色KF / L2-09 Speed分段 / L2-10 KFToggle门控（2612c68 + 前批）
- C组2：L2-01 Blend 融合 / L2-18 替换素材（16eb450）
- D组1：L2-23 拖素材清空/回弹根治=B-01/B-03 同源乐观锁竞态（1eee1c2）
- 状态统一「代码已落·待真机验收」；C列写可测验收标准（含依赖/红线标注）；E列标注 commit + L0-07/L0-08 合规
- 同步桌面副本 C:/Users/34450/Desktop/git-commit-log.xlsx
</commit_message>
<xml_diff>
--- a/docs/git-commit-log.xlsx
+++ b/docs/git-commit-log.xlsx
@@ -3146,7 +3146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="3" min="1" max="1"/>
@@ -5236,6 +5236,313 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>L2-01</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>1. 选中 video/image 段 → 属性面板出现「融合」tab；下拉含 16 项中文（正常/正片叠底/滤色/叠加/变暗/变亮/颜色减淡/颜色加深/柔光/强光/差值/排除/色相/饱和度/颜色/明度）。
+2. 切换融合模式 → 预览画面实时混合变化；旧草稿默认 normal 回退正常。
+3. 切换后 undo 一次可恢复上一模式。
+4. 文本/音频段不出现融合 tab（仅 video/image 可设）。
+5. 落库：段内 blend_mode 字段写入；get_state 可见；重开草稿保留。</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>C组 已提交 16eb450；blend 段内字段经 set_segments_props 白名单（对齐 speed 先例，零新增Api）；不做KF；🔴L0-07合规</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>L2-02</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>1. 选中文本段 → 属性面板「样式」tab 可编辑字号/字距/行距/粗体/颜色。
+2. 改样式 → 预览实时更新（提交后落库）。
+3. 字号/字距/颜色通道 ◆ 可打帧：播放头在段内点 ◆ → 写入 text.fontSize 等通道关键帧；段外 ◆ 禁用（L2-10 门控）。
+4. 粗体(discrete 布尔通道) → 取左帧值（两帧间不插值）。
+5. 颜色 KF 走四分量 text.color.r/g/b/a，红→蓝平滑过渡（与 L2-07 同机制）。
+6. 撤销：样式改 + 打帧各记一条 undo。</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>A组 已提交 2612c68；KF_KEYFRAMEABLE 白名单追加文本path+discrete bool；value 放行 bool/str(docstring)；🔴L0-07/L0-08 Q1=A</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>L2-04</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>1. 工具栏「图形」按钮 → 在时间轴 text 轨当前播放头处新建 graphic 段（圆角矩形，默认描边+填充）。
+2. 选中 graphic 段 → 「图形」tab：描边开关/宽度/颜色、填充颜色、圆角，均可编辑实时预览。
+3. 描边宽度/颜色/圆角/填充色 ◆ 可打帧（params.stroke.width / params.fill.color.* / params.radius），播放头在段内写入通道。
+4. 字幕查询 get_track_text 不返回 graphic 段（语义裁剪，🔴L0-07 合规）。
+5. 旧草稿无 graphic 段 → 兼容正常加载。</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>A组 已提交 2612c68；graphic 段挂 text 轨(track_type 三枚举不动)；add_graphic 经 getattr 可被 call 调；params.* 进 KF_KEYFRAMEABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>L2-05</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="inlineStr">
+        <is>
+          <t>1. 选中含 ≥2 个关键帧的属性通道 → KF 面板出现 Graph Editor 按钮/Popover。
+2. 拖贝塞尔控制柄 → 曲线实时变化，提交一条 undo。
+3. 6 预设（ease/linear/ease-in/out/in-out/…）一键应用。
+4. 缓动写入 keys 四字段（L0-08 Q1=A 追加），重开草稿保留。
+5. 无缓动属性（静态/单帧）不出现 Graph Editor。</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E64" s="18" t="inlineStr">
+        <is>
+          <t>A组 已提交 d14bf9c(前批)；graph-editor.js + main.py bezier 分支；追加可选参不碰签名；🔴L0-08 Q1=A</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>L2-06</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>1. 选中带 transform 的段 → KF 面板 Scale 组有「锁形」按钮。
+2. 锁定后 W/H 合成单 Scale 字段 + 成组菱形；改一处等比双写。
+3. 成组菱形同 t 同增删（一次 upsert 两条通道）。
+4. 解锁后恢复独立 W/H 通道。</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>A组 已提交(前批)；纯前端复用 add/remove_keyframe，Api 不碰</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>L2-07</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="inlineStr">
+        <is>
+          <t>1. 颜色属性（文本色/填充色/描边色）出现 ColorPicker 组件（非原生 input）。
+2. 色块 Popover 拖动 → 预览实时；◆ 打四条同 t 通道（r/g/b/a）。
+3. 红→蓝关键帧间平滑过渡（四分量各自插值）。
+4. 四分量合并单 ◆（对齐 L2-02 文本色机制），path 前缀可配。</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E66" s="18" t="inlineStr">
+        <is>
+          <t>A组 已提交 2bf9030(前批)；KF_KEYFRAMEABLE 追加 text.color.r/g/b/a；复用 add/remove_keyframe；🔴L0-08 Q1=A</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>L2-09</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="inlineStr">
+        <is>
+          <t>1. speed 字段左侧 icon 改为可拖 scrub 手柄（指针锁定 Pointer Lock）。
+2. 两段灵敏度：粗调段 + 精调段（实时预览一条 undo）。
+3. 批量选中 2+ 段 → 同步 scrub。
+4. ⚠ 依赖层1 L1-17 drag-to-scrub 手势（L1-17 当前阻塞·待用户决策）；若 L1-17 未落，scrub 手柄交互可能未完全生效，验收时标注。</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E67" s="18" t="inlineStr">
+        <is>
+          <t>A组 已提交(前批)；speed-panel.js scrub 手柄；复用 set_segment_speed；依赖 L1-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>L2-10</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>1. 播放头在段范围内 → ◆ 实心可点（inRange 态）。
+2. 播放头出段范围 → ◆ 灰禁 + opacity.5，点击无效（禁用态）。
+3. 段外改输入值 → 只落 base（不打帧）。
+4. ±1 帧内命中 → 删除该关键帧。</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E68" s="18" t="inlineStr">
+        <is>
+          <t>A组 已提交(前批)；timeline-mapper.js isPlayheadWithinRange + kf-panel 第三态；门控语义由 L0-06 定义</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>L2-18</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>1. 素材库同类型素材（video→video / image→image）拖到时间轴已有段上 → 就地换源（非删建）。
+2. 换源后段 id 不变（撤销栈/选中/动画/特效绑定不断裂）。
+3. duration 重置为新素材全长（src_start/src_end/src_full 同步）。
+4. 换源后 undo 一次恢复旧源。
+5. 跨类型（video→image）拖入不触发替换（走正常新增或忽略）。</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="inlineStr">
+        <is>
+          <t>C组 已提交 16eb450；replace_segment_source 加性Api(分支B 段id稳定)；🔴L0-07复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>L2-23</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>1. 单段拖素材入轨 → 段正常落盘，不回弹（B-01 拖入回弹不再现）。
+2. 快速连续拖入多段 → 无段丢失/清空（B-03 拖入清空不再现）。
+3. 并发拖入（前端串行化队列 + 后端乐观锁冲突重试最多5次）→ 段全部落盘、id 稳定。
+4. 后端 SAVE_LAST_CONFLICT 记录冲突重试过程（控制台可见），前端不再静默丢段。
+5. 回归：refresh() 空稿防御 + isLibraryDragging 并入 refresh Lock（拖入中不被轮询刷新覆盖）。</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="inlineStr">
+        <is>
+          <t>D组 已提交 1eee1c2；根因=save_state 乐观锁冲突被当成功(非空dict真值)，改 return False + add_to_timeline 重试 + 前端__addChain 串行化；B-01/B-03 同源根治</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
R3/L1-17: drag-to-scrub 全参数数字字段（共享 ScrubSession）
新建 property/scrub-session.js（ScrubSession+attachScrub+scrubAcrossRanges），复用 InteractionKernel 单会话互斥 + refresh 锁（previewActive 已查 InteractionManager.blocksRefresh）；Pointer Lock 拖动、首帧 movementX 跳过、onScrub→preview(实时不落库)/onScrubEnd→commit(一条undo)/Esc→onCancel(回退起始值)。NumberField 加通用 scrub icon（类当前未实例化，未来字段自动带）；speed/audio/kf 三面板数字字段（⏩/🔊/⇔）全部接入，KF 走 L0-06 门控（有通道范围→打点 overlay，无→base）。speed-panel 内联 scrub 重构为共享（消除 L2-09 双份）+ 移除 _scrubbing 守卫。验收两表 L1-17(R30) 状态更新为「代码已落·待真机验收」，顺手修 L1-14 差距表不一致。红线未破：不碰 Api/draft schema/seg_id/track_type/MCP/player/Video DSL。
</commit_message>
<xml_diff>
--- a/docs/git-commit-log.xlsx
+++ b/docs/git-commit-log.xlsx
@@ -1974,17 +1974,17 @@
       </c>
       <c r="E27" s="27" t="inlineStr">
         <is>
-          <t>未落（按分支A：前置后端 update_text，本论前端不做）</t>
+          <t>已落：text-edit-overlay.js + window.__textEditing 守卫（commit 598c831）</t>
         </is>
       </c>
       <c r="F27" s="27" t="inlineStr">
         <is>
-          <t>阻塞·待用户决策</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G27" s="27" t="inlineStr">
         <is>
-          <t>需后端补 update_text 命令后再收口</t>
+          <t>后端零新增 Api（text 白名单已就位）；与验收总表 R27 对齐</t>
         </is>
       </c>
     </row>
@@ -2085,17 +2085,17 @@
       </c>
       <c r="E30" s="27" t="inlineStr">
         <is>
-          <t>未落（本次未实现，标阻塞待决策）</t>
+          <t>已落：scrub-session.js 新建 + speed/audio/kf-panel 三处接入 attachScrub；commit 待补</t>
         </is>
       </c>
       <c r="F30" s="27" t="inlineStr">
         <is>
-          <t>阻塞·待用户决策</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G30" s="27" t="inlineStr">
         <is>
-          <t>需立项 ScrubSession 前端新增（较大）</t>
+          <t>共享 ScrubSession 收口 L2-09 内联双份；L0-03 预览态已落地→原阻塞理由失效；Pointer Lock WebView2 已验证；与 L1-14 同批 commit。</t>
         </is>
       </c>
     </row>
@@ -4130,12 +4130,12 @@
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>阻塞·待用户决策</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E30" s="27" t="inlineStr">
         <is>
-          <t>需立项 ScrubSession 前端新增（较大）</t>
+          <t>已落：新建 property/scrub-session.js（共享 ScrubSession extends GestureSession + attachScrub + scrubAcrossRanges），复用 InteractionKernel 单会话互斥 + refresh 锁（previewActive 已查 InteractionManager.blocksRefresh）。speed/audio/kf-panel 三面板数字字段全部接入 drag-to-scrub（⏩/🔊/⇔ 把手）：onScrub→preview 实时不落库、onScrubEnd→commit 一条 undo、Esc/pointercancel→onCancel 回退起始值；Pointer Lock 在 L2-09 已验证可用，首帧 movementX 跳过。NumberField 类亦加通用 icon（当前未实例化，未来字段自动带把手）。原“缺 L0-03”阻塞理由已失效（L0-03 preview-state 已落地 ba87c96）；红线未破。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
R3 修复 L2-04/17/23 真缺口 + DRIFT纠正 L2-24/26/27 误判
- L2-04: mcp_server.py 6处 sr.->api.(list_tracks/get_track_text/get_segment_detail/get_effects/get_material_peaks/get_segment_peaks 因 sr 未定义必崩)；main.py 实现6个只读方法(纯读,M1安全线)
- L2-17: main.py import_media_by_paths 入仓项加 duration_for(dst,mtype) 加性字段(微秒)，前端时长徽标不再空转
- L2-23: refresh() 加 _refreshSeq 乱序串行化 + #516-guard 空稿防御(A-1/A-2)，只挡读盘竞态半写文件，合法空库不受影响
- L2-26: TRACK_H=48 死常量注释澄清(实际逐类型高度由 trackHeightOf 计算)
- DRIFT纠正: L2-24/26/27 原判未达标源于读卡片①现状陈旧快照，真实代码已落码，纠正为代码已落·待真机验收
- 验收报告 R3-整体验收报告-2026-08-28.md 加第六节纠正；xlsx 验收差距表/验收总表同步
</commit_message>
<xml_diff>
--- a/docs/git-commit-log.xlsx
+++ b/docs/git-commit-log.xlsx
@@ -977,7 +977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="3" min="1" max="1"/>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="F2" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G2" s="27" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="F3" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G3" s="27" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F4" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G4" s="27" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="F5" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G5" s="27" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="F6" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G6" s="27" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="F7" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="F8" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G8" s="27" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="F9" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="F10" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G10" s="27" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="F11" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G11" s="27" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="F12" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G12" s="27" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="F13" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G13" s="27" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="F14" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G14" s="27" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="F15" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G15" s="27" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="F16" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G16" s="27" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="F17" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G17" s="27" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="F18" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G18" s="27" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="F19" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G19" s="27" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="F20" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G20" s="27" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="F21" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G21" s="27" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="F22" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G22" s="27" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="F23" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G23" s="27" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="F24" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G24" s="27" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F25" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G25" s="27" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="F26" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G26" s="27" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="F28" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G28" s="27" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="F29" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G29" s="27" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="F31" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G31" s="27" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="F32" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G32" s="27" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="F33" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G33" s="27" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="F34" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G34" s="27" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="F35" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G35" s="27" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="F36" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G36" s="27" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="F37" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G37" s="27" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
@@ -2529,17 +2529,17 @@
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>commit e9e9e82（纯前端，不碰 Api/draft schema/seg_id/track_type/MCP/player/Video DSL）</t>
+          <t>— 未动</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>待决·设计未裁定(未动)</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>行为需真机验收</t>
+          <t>段级音量已落；控制条独立音量滑块+loop 属 Q9 未裁定（分支B可不纳入）</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
@@ -2677,17 +2677,17 @@
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>commit 94b9b8d（纯前端，不碰 Api/draft schema/seg_id/track_type/MCP/player/Video DSL）</t>
+          <t>修 main.py import_media_by_paths 入仓项加 duration_for(dst,mtype)（加性字段,微秒）</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>数据源 m.duration 挂起 L0-07 裁定；徽标基建完成，数据到位即亮</t>
+          <t>前端徽标CSS(HTML:158-160)已落；补数据源后徽标不再空转</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2719,7 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
@@ -2862,17 +2862,17 @@
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>commit c286b6d（纯前端，不碰 Api/draft schema/seg_id/track_type/MCP/player/Video DSL）</t>
+          <t>— DRIFT纠正：实际已落</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>行为需真机验收</t>
+          <t>timeline.js:602-604(keyed-diff)+:714-716(全量) 注入 track-selected + HTML:488-489 CSS，原判误读卡片①快照</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2904,7 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
@@ -2936,17 +2936,17 @@
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>commit c286b6d（纯前端，不碰 Api/draft schema/seg_id/track_type/MCP/player/Video DSL）</t>
+          <t>— DRIFT纠正：实际已落</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>行为需真机验收</t>
+          <t>timeline.js:404-413 trackHeightOf()+HTML 逐类型CSS/6px间距已落；TRACK_H=48仅剩回退常量</t>
         </is>
       </c>
     </row>
@@ -2973,17 +2973,17 @@
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>commit 25c05f2（纯前端，不碰 Api/draft schema/seg_id/track_type/MCP/player/Video DSL）</t>
+          <t>— DRIFT纠正：KF 40px 门限已落</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>行为需真机验收</t>
+          <t>timeline.js:526-529 if(segWidthPx&lt;40) continue；其余10子项按真机核验</t>
         </is>
       </c>
     </row>
@@ -3015,7 +3015,7 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
@@ -3126,12 +3126,123 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>接口预留·未启用</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
           <t>Q11 未裁定，只留接口不启用</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>L2-04</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>未达标(原判)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Graphic/get_track_text：mcp_server sr未定义必崩 + 后端缺6只读方法</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>修 sr-&gt;api(6工具) + main.py 实现 list_tracks/get_track_text/get_segment_detail/get_effects/get_material_peaks/get_segment_peaks</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>DRIFT纠正：原判误读卡片①快照；sr真缺口本轮已修</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>L2-05</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>未达标(原判)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Graph Editor Saved 自定义曲线保存/删除未实现</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>— 未动</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>待决·设计未裁定(未动)</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>整编辑器依赖 L0-08 Q1 数据层裁决，属大特性</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>L2-23</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>层2</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>未达标(原判)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>拖素材清空bug：空稿防御+乱序刷新串行化缺失</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>修 refresh() 加 _refreshSeq 串行化 + #516-guard 空稿防御(A-1/A-2)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>代码已落·待真机验收</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>只挡读盘竞态半写文件，合法空库不受影响</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3318,7 @@
       </c>
       <c r="D2" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E2" s="27" t="inlineStr">
@@ -3240,7 +3351,7 @@
       </c>
       <c r="D3" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E3" s="27" t="inlineStr">
@@ -3273,7 +3384,7 @@
       </c>
       <c r="D4" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E4" s="27" t="inlineStr">
@@ -3306,7 +3417,7 @@
       </c>
       <c r="D5" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E5" s="27" t="inlineStr">
@@ -3339,7 +3450,7 @@
       </c>
       <c r="D6" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr">
@@ -3371,7 +3482,7 @@
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
@@ -3404,7 +3515,7 @@
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
@@ -3437,7 +3548,7 @@
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr">
@@ -3470,7 +3581,7 @@
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr">
@@ -3503,7 +3614,7 @@
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E11" s="27" t="inlineStr">
@@ -3537,7 +3648,7 @@
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr">
@@ -3570,7 +3681,7 @@
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E13" s="27" t="inlineStr">
@@ -3603,7 +3714,7 @@
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr">
@@ -3636,7 +3747,7 @@
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E15" s="27" t="inlineStr">
@@ -3670,7 +3781,7 @@
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
@@ -3703,7 +3814,7 @@
       </c>
       <c r="D17" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
@@ -3735,7 +3846,7 @@
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
@@ -3769,7 +3880,7 @@
       </c>
       <c r="D19" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E19" s="27" t="inlineStr">
@@ -3801,7 +3912,7 @@
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E20" s="27" t="inlineStr">
@@ -3833,7 +3944,7 @@
       </c>
       <c r="D21" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
@@ -3865,7 +3976,7 @@
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E22" s="27" t="inlineStr">
@@ -3898,7 +4009,7 @@
       </c>
       <c r="D23" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E23" s="27" t="inlineStr">
@@ -3931,7 +4042,7 @@
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>机制落地</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E24" s="27" t="inlineStr">
@@ -3964,7 +4075,7 @@
       </c>
       <c r="D25" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E25" s="27" t="inlineStr">
@@ -3997,7 +4108,7 @@
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
@@ -4063,7 +4174,7 @@
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E28" s="27" t="inlineStr">
@@ -4096,7 +4207,7 @@
       </c>
       <c r="D29" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E29" s="27" t="inlineStr">
@@ -4163,7 +4274,7 @@
       </c>
       <c r="D31" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E31" s="27" t="inlineStr">
@@ -4196,7 +4307,7 @@
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E32" s="27" t="inlineStr">
@@ -4229,7 +4340,7 @@
       </c>
       <c r="D33" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E33" s="27" t="inlineStr">
@@ -4262,7 +4373,7 @@
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E34" s="27" t="inlineStr">
@@ -4295,7 +4406,7 @@
       </c>
       <c r="D35" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E35" s="27" t="inlineStr">
@@ -4330,7 +4441,7 @@
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E36" s="27" t="inlineStr">
@@ -4363,7 +4474,7 @@
       </c>
       <c r="D37" s="27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>代码已落·待真机验收</t>
         </is>
       </c>
       <c r="E37" s="27" t="inlineStr">
@@ -4594,7 +4705,7 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>代码已落·待真机验收</t>
+          <t>待决·需Q9裁定</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -5227,7 +5338,7 @@
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>代码已落·待真机验收</t>
+          <t>接口预留·未启用</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -5352,7 +5463,7 @@
       </c>
       <c r="D64" s="18" t="inlineStr">
         <is>
-          <t>代码已落·待真机验收</t>
+          <t>待决·需L0-08 Q1裁决</t>
         </is>
       </c>
       <c r="E64" s="18" t="inlineStr">

</xml_diff>